<commit_message>
South & Southeast Asia pulls: branch run
</commit_message>
<xml_diff>
--- a/output/Data and Chart Outputs/india_coal_stocks.xlsx
+++ b/output/Data and Chart Outputs/india_coal_stocks.xlsx
@@ -28673,7 +28673,7 @@
         <v>225187.5</v>
       </c>
       <c r="G819" t="n">
-        <v>8.5</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="820">
@@ -28696,7 +28696,7 @@
         <v>225187.5</v>
       </c>
       <c r="G820" t="n">
-        <v>8.300000000000001</v>
+        <v>7.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>